<commit_message>
Funde aluna duplicada no comparativo e adiciona analise de itens
A 11a Fase aparecia com "Maria Amelia Vozniak Deluca" no Simulado 01 e
"Maria Amelia Vozniak Deluca Schneider" no Simulado 02 - mesma aluna,
sobrenome cortado na primeira imagem. Sem a fusao ela contava como dois
alunos e ficava fora do comparativo (agora 113 alunos nos dois simulados).

Acrescenta analise.py: formato dos itens, dificuldade, progressao entre
fases, itens em que um distrator vence o gabarito e distratores nao
funcionais.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KJtXaVvEGRV3wqA1hqbBYb
</commit_message>
<xml_diff>
--- a/dados/Dados_Simulados_MED_ENAMED_2026.xlsx
+++ b/dados/Dados_Simulados_MED_ENAMED_2026.xlsx
@@ -21,7 +21,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Questão x Fase'!$A$1:$H$401</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Distribuição respostas'!$A$1:$H$1769</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Resumo por fase'!$A$1:$K$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Comparativo S01 x S02'!$A$1:$H$127</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Comparativo S01 x S02'!$A$1:$H$126</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -655,7 +655,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="26" customHeight="1">
+    <row r="12" ht="91" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Ressalva 4 — nomes</t>
@@ -663,7 +663,7 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Dois nomes apareciam truncados na imagem da 10ª Fase do Simulado 01 ('Lucas Eduardo dos Santos Vian…' e 'Maria Eduarda Medeiros Macha…'); foram completados pela lista do Simulado 02.</t>
+          <t>Os 126 nomes foram lidos duas vezes de forma independente (uma imagem por simulado) e 112 coincidem caractere a caractere, o que confirma essa leitura. Três casos exigiram intervenção: 'Lucas Eduardo dos Santos Vian…' e 'Maria Eduarda Medeiros Macha…' estavam truncados na imagem da 10ª Fase do Simulado 01 e foram completados pela lista do Simulado 02; e 'Maria Amélia Vozniak Deluca' (S01) e 'Maria Amélia Vozniak Deluca Schneider' (S02) são a mesma aluna, unificadas na aba de comparativo. Os 13 nomes restantes que aparecem em um só simulado são mudanças reais de turma (a 11ª Fase perdeu 4 alunos e ganhou 6 entre as duas aplicações).</t>
         </is>
       </c>
     </row>
@@ -92005,7 +92005,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H127"/>
+  <dimension ref="A1:H126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -94913,7 +94913,7 @@
     <row r="84">
       <c r="A84" s="7" t="inlineStr">
         <is>
-          <t>Maria Amélia Vozniak Deluca</t>
+          <t>Maria Amélia Vozniak Deluca Schneider</t>
         </is>
       </c>
       <c r="B84" s="8" t="inlineStr">
@@ -94928,7 +94928,9 @@
         <f>IF(C84="","",C84/39)</f>
         <v/>
       </c>
-      <c r="E84" s="8" t="n"/>
+      <c r="E84" s="8" t="n">
+        <v>38</v>
+      </c>
       <c r="F84" s="9">
         <f>IF(E84="","",E84/60)</f>
         <v/>
@@ -94939,28 +94941,30 @@
       </c>
       <c r="H84" s="7" t="inlineStr">
         <is>
-          <t>Só no Simulado 01</t>
+          <t>Nos dois simulados</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="10" t="inlineStr">
         <is>
-          <t>Maria Amélia Vozniak Deluca Schneider</t>
+          <t>Maria Eduarda Medeiros Machado</t>
         </is>
       </c>
       <c r="B85" s="11" t="inlineStr">
         <is>
-          <t>11ª Fase</t>
-        </is>
-      </c>
-      <c r="C85" s="11" t="n"/>
+          <t>10ª Fase</t>
+        </is>
+      </c>
+      <c r="C85" s="11" t="n">
+        <v>26</v>
+      </c>
       <c r="D85" s="12">
         <f>IF(C85="","",C85/39)</f>
         <v/>
       </c>
       <c r="E85" s="11" t="n">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="F85" s="12">
         <f>IF(E85="","",E85/60)</f>
@@ -94972,14 +94976,14 @@
       </c>
       <c r="H85" s="10" t="inlineStr">
         <is>
-          <t>Só no Simulado 02</t>
+          <t>Nos dois simulados</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="7" t="inlineStr">
         <is>
-          <t>Maria Eduarda Medeiros Machado</t>
+          <t>Maria Eduarda Molinari</t>
         </is>
       </c>
       <c r="B86" s="8" t="inlineStr">
@@ -94988,14 +94992,14 @@
         </is>
       </c>
       <c r="C86" s="8" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D86" s="9">
         <f>IF(C86="","",C86/39)</f>
         <v/>
       </c>
       <c r="E86" s="8" t="n">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="F86" s="9">
         <f>IF(E86="","",E86/60)</f>
@@ -95014,23 +95018,23 @@
     <row r="87">
       <c r="A87" s="10" t="inlineStr">
         <is>
-          <t>Maria Eduarda Molinari</t>
+          <t>Maria Eduarda Silveira Navarro Lins</t>
         </is>
       </c>
       <c r="B87" s="11" t="inlineStr">
         <is>
-          <t>10ª Fase</t>
+          <t>6ª Fase</t>
         </is>
       </c>
       <c r="C87" s="11" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D87" s="12">
         <f>IF(C87="","",C87/39)</f>
         <v/>
       </c>
       <c r="E87" s="11" t="n">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="F87" s="12">
         <f>IF(E87="","",E87/60)</f>
@@ -95049,7 +95053,7 @@
     <row r="88">
       <c r="A88" s="7" t="inlineStr">
         <is>
-          <t>Maria Eduarda Silveira Navarro Lins</t>
+          <t>Maria Isadora Baptista Pianezzer</t>
         </is>
       </c>
       <c r="B88" s="8" t="inlineStr">
@@ -95058,14 +95062,14 @@
         </is>
       </c>
       <c r="C88" s="8" t="n">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="D88" s="9">
         <f>IF(C88="","",C88/39)</f>
         <v/>
       </c>
       <c r="E88" s="8" t="n">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="F88" s="9">
         <f>IF(E88="","",E88/60)</f>
@@ -95084,23 +95088,23 @@
     <row r="89">
       <c r="A89" s="10" t="inlineStr">
         <is>
-          <t>Maria Isadora Baptista Pianezzer</t>
+          <t>Maria Luísa Ceolin Xavier da Silveira</t>
         </is>
       </c>
       <c r="B89" s="11" t="inlineStr">
         <is>
-          <t>6ª Fase</t>
+          <t>7ª Fase</t>
         </is>
       </c>
       <c r="C89" s="11" t="n">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="D89" s="12">
         <f>IF(C89="","",C89/39)</f>
         <v/>
       </c>
       <c r="E89" s="11" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F89" s="12">
         <f>IF(E89="","",E89/60)</f>
@@ -95119,23 +95123,23 @@
     <row r="90">
       <c r="A90" s="7" t="inlineStr">
         <is>
-          <t>Maria Luísa Ceolin Xavier da Silveira</t>
+          <t>Mariana Braatz Fagundes</t>
         </is>
       </c>
       <c r="B90" s="8" t="inlineStr">
         <is>
-          <t>7ª Fase</t>
+          <t>10ª Fase</t>
         </is>
       </c>
       <c r="C90" s="8" t="n">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="D90" s="9">
         <f>IF(C90="","",C90/39)</f>
         <v/>
       </c>
       <c r="E90" s="8" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F90" s="9">
         <f>IF(E90="","",E90/60)</f>
@@ -95154,7 +95158,7 @@
     <row r="91">
       <c r="A91" s="10" t="inlineStr">
         <is>
-          <t>Mariana Braatz Fagundes</t>
+          <t>Marieva Niehues Anderle</t>
         </is>
       </c>
       <c r="B91" s="11" t="inlineStr">
@@ -95163,14 +95167,14 @@
         </is>
       </c>
       <c r="C91" s="11" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D91" s="12">
         <f>IF(C91="","",C91/39)</f>
         <v/>
       </c>
       <c r="E91" s="11" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F91" s="12">
         <f>IF(E91="","",E91/60)</f>
@@ -95189,23 +95193,23 @@
     <row r="92">
       <c r="A92" s="7" t="inlineStr">
         <is>
-          <t>Marieva Niehues Anderle</t>
+          <t>Mateus Henrique Silva</t>
         </is>
       </c>
       <c r="B92" s="8" t="inlineStr">
         <is>
-          <t>10ª Fase</t>
+          <t>11ª Fase</t>
         </is>
       </c>
       <c r="C92" s="8" t="n">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="D92" s="9">
         <f>IF(C92="","",C92/39)</f>
         <v/>
       </c>
       <c r="E92" s="8" t="n">
-        <v>34</v>
+        <v>54</v>
       </c>
       <c r="F92" s="9">
         <f>IF(E92="","",E92/60)</f>
@@ -95224,23 +95228,23 @@
     <row r="93">
       <c r="A93" s="10" t="inlineStr">
         <is>
-          <t>Mateus Henrique Silva</t>
+          <t>Matheus Lazzarin Gramazio</t>
         </is>
       </c>
       <c r="B93" s="11" t="inlineStr">
         <is>
-          <t>11ª Fase</t>
+          <t>10ª Fase</t>
         </is>
       </c>
       <c r="C93" s="11" t="n">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="D93" s="12">
         <f>IF(C93="","",C93/39)</f>
         <v/>
       </c>
       <c r="E93" s="11" t="n">
-        <v>54</v>
+        <v>40</v>
       </c>
       <c r="F93" s="12">
         <f>IF(E93="","",E93/60)</f>
@@ -95259,7 +95263,7 @@
     <row r="94">
       <c r="A94" s="7" t="inlineStr">
         <is>
-          <t>Matheus Lazzarin Gramazio</t>
+          <t>Matheus Schmidt Rossini</t>
         </is>
       </c>
       <c r="B94" s="8" t="inlineStr">
@@ -95275,7 +95279,7 @@
         <v/>
       </c>
       <c r="E94" s="8" t="n">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="F94" s="9">
         <f>IF(E94="","",E94/60)</f>
@@ -95294,23 +95298,23 @@
     <row r="95">
       <c r="A95" s="10" t="inlineStr">
         <is>
-          <t>Matheus Schmidt Rossini</t>
+          <t>Maísa Laguna</t>
         </is>
       </c>
       <c r="B95" s="11" t="inlineStr">
         <is>
-          <t>10ª Fase</t>
+          <t>6ª Fase</t>
         </is>
       </c>
       <c r="C95" s="11" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D95" s="12">
         <f>IF(C95="","",C95/39)</f>
         <v/>
       </c>
       <c r="E95" s="11" t="n">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="F95" s="12">
         <f>IF(E95="","",E95/60)</f>
@@ -95329,23 +95333,23 @@
     <row r="96">
       <c r="A96" s="7" t="inlineStr">
         <is>
-          <t>Maísa Laguna</t>
+          <t>Micheli Padilha</t>
         </is>
       </c>
       <c r="B96" s="8" t="inlineStr">
         <is>
-          <t>6ª Fase</t>
+          <t>11ª Fase</t>
         </is>
       </c>
       <c r="C96" s="8" t="n">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="D96" s="9">
         <f>IF(C96="","",C96/39)</f>
         <v/>
       </c>
       <c r="E96" s="8" t="n">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="F96" s="9">
         <f>IF(E96="","",E96/60)</f>
@@ -95364,23 +95368,23 @@
     <row r="97">
       <c r="A97" s="10" t="inlineStr">
         <is>
-          <t>Micheli Padilha</t>
+          <t>Milena Ferreira de Souza</t>
         </is>
       </c>
       <c r="B97" s="11" t="inlineStr">
         <is>
-          <t>11ª Fase</t>
+          <t>7ª Fase</t>
         </is>
       </c>
       <c r="C97" s="11" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="D97" s="12">
         <f>IF(C97="","",C97/39)</f>
         <v/>
       </c>
       <c r="E97" s="11" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="F97" s="12">
         <f>IF(E97="","",E97/60)</f>
@@ -95399,7 +95403,7 @@
     <row r="98">
       <c r="A98" s="7" t="inlineStr">
         <is>
-          <t>Milena Ferreira de Souza</t>
+          <t>Milena Goedert</t>
         </is>
       </c>
       <c r="B98" s="8" t="inlineStr">
@@ -95408,14 +95412,14 @@
         </is>
       </c>
       <c r="C98" s="8" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D98" s="9">
         <f>IF(C98="","",C98/39)</f>
         <v/>
       </c>
       <c r="E98" s="8" t="n">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F98" s="9">
         <f>IF(E98="","",E98/60)</f>
@@ -95434,16 +95438,16 @@
     <row r="99">
       <c r="A99" s="10" t="inlineStr">
         <is>
-          <t>Milena Goedert</t>
+          <t>Milena Marchi Bonacolsi</t>
         </is>
       </c>
       <c r="B99" s="11" t="inlineStr">
         <is>
-          <t>7ª Fase</t>
+          <t>10ª Fase</t>
         </is>
       </c>
       <c r="C99" s="11" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D99" s="12">
         <f>IF(C99="","",C99/39)</f>
@@ -95469,23 +95473,23 @@
     <row r="100">
       <c r="A100" s="7" t="inlineStr">
         <is>
-          <t>Milena Marchi Bonacolsi</t>
+          <t>Millena Laurindo</t>
         </is>
       </c>
       <c r="B100" s="8" t="inlineStr">
         <is>
-          <t>10ª Fase</t>
+          <t>7ª Fase</t>
         </is>
       </c>
       <c r="C100" s="8" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D100" s="9">
         <f>IF(C100="","",C100/39)</f>
         <v/>
       </c>
       <c r="E100" s="8" t="n">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="F100" s="9">
         <f>IF(E100="","",E100/60)</f>
@@ -95504,16 +95508,16 @@
     <row r="101">
       <c r="A101" s="10" t="inlineStr">
         <is>
-          <t>Millena Laurindo</t>
+          <t>Nicoly Fiorese Andrade</t>
         </is>
       </c>
       <c r="B101" s="11" t="inlineStr">
         <is>
-          <t>7ª Fase</t>
+          <t>10ª Fase</t>
         </is>
       </c>
       <c r="C101" s="11" t="n">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="D101" s="12">
         <f>IF(C101="","",C101/39)</f>
@@ -95539,16 +95543,16 @@
     <row r="102">
       <c r="A102" s="7" t="inlineStr">
         <is>
-          <t>Nicoly Fiorese Andrade</t>
+          <t>Pedro Henrique Daniel Abreu</t>
         </is>
       </c>
       <c r="B102" s="8" t="inlineStr">
         <is>
-          <t>10ª Fase</t>
+          <t>6ª Fase</t>
         </is>
       </c>
       <c r="C102" s="8" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D102" s="9">
         <f>IF(C102="","",C102/39)</f>
@@ -95574,7 +95578,7 @@
     <row r="103">
       <c r="A103" s="10" t="inlineStr">
         <is>
-          <t>Pedro Henrique Daniel Abreu</t>
+          <t>Pedro Werner Eger</t>
         </is>
       </c>
       <c r="B103" s="11" t="inlineStr">
@@ -95583,14 +95587,14 @@
         </is>
       </c>
       <c r="C103" s="11" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D103" s="12">
         <f>IF(C103="","",C103/39)</f>
         <v/>
       </c>
       <c r="E103" s="11" t="n">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="F103" s="12">
         <f>IF(E103="","",E103/60)</f>
@@ -95609,23 +95613,23 @@
     <row r="104">
       <c r="A104" s="7" t="inlineStr">
         <is>
-          <t>Pedro Werner Eger</t>
+          <t>Rafaela Dela Justina</t>
         </is>
       </c>
       <c r="B104" s="8" t="inlineStr">
         <is>
-          <t>6ª Fase</t>
+          <t>11ª Fase</t>
         </is>
       </c>
       <c r="C104" s="8" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="D104" s="9">
         <f>IF(C104="","",C104/39)</f>
         <v/>
       </c>
       <c r="E104" s="8" t="n">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="F104" s="9">
         <f>IF(E104="","",E104/60)</f>
@@ -95644,7 +95648,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Rafaela Dela Justina</t>
+          <t>Ramon Hüntermann</t>
         </is>
       </c>
       <c r="B105" s="11" t="inlineStr">
@@ -95653,14 +95657,14 @@
         </is>
       </c>
       <c r="C105" s="11" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D105" s="12">
         <f>IF(C105="","",C105/39)</f>
         <v/>
       </c>
       <c r="E105" s="11" t="n">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="F105" s="12">
         <f>IF(E105="","",E105/60)</f>
@@ -95679,7 +95683,7 @@
     <row r="106">
       <c r="A106" s="7" t="inlineStr">
         <is>
-          <t>Ramon Hüntermann</t>
+          <t>Raquel Michels</t>
         </is>
       </c>
       <c r="B106" s="8" t="inlineStr">
@@ -95688,14 +95692,14 @@
         </is>
       </c>
       <c r="C106" s="8" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D106" s="9">
         <f>IF(C106="","",C106/39)</f>
         <v/>
       </c>
       <c r="E106" s="8" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F106" s="9">
         <f>IF(E106="","",E106/60)</f>
@@ -95714,23 +95718,23 @@
     <row r="107">
       <c r="A107" s="10" t="inlineStr">
         <is>
-          <t>Raquel Michels</t>
+          <t>Rodrigo Voigt Filho</t>
         </is>
       </c>
       <c r="B107" s="11" t="inlineStr">
         <is>
-          <t>11ª Fase</t>
+          <t>7ª Fase</t>
         </is>
       </c>
       <c r="C107" s="11" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D107" s="12">
         <f>IF(C107="","",C107/39)</f>
         <v/>
       </c>
       <c r="E107" s="11" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="F107" s="12">
         <f>IF(E107="","",E107/60)</f>
@@ -95749,23 +95753,23 @@
     <row r="108">
       <c r="A108" s="7" t="inlineStr">
         <is>
-          <t>Rodrigo Voigt Filho</t>
+          <t>Sanny Machado</t>
         </is>
       </c>
       <c r="B108" s="8" t="inlineStr">
         <is>
-          <t>7ª Fase</t>
+          <t>10ª Fase</t>
         </is>
       </c>
       <c r="C108" s="8" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D108" s="9">
         <f>IF(C108="","",C108/39)</f>
         <v/>
       </c>
       <c r="E108" s="8" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F108" s="9">
         <f>IF(E108="","",E108/60)</f>
@@ -95784,7 +95788,7 @@
     <row r="109">
       <c r="A109" s="10" t="inlineStr">
         <is>
-          <t>Sanny Machado</t>
+          <t>Sofia Boldrini</t>
         </is>
       </c>
       <c r="B109" s="11" t="inlineStr">
@@ -95793,14 +95797,14 @@
         </is>
       </c>
       <c r="C109" s="11" t="n">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="D109" s="12">
         <f>IF(C109="","",C109/39)</f>
         <v/>
       </c>
       <c r="E109" s="11" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F109" s="12">
         <f>IF(E109="","",E109/60)</f>
@@ -95819,23 +95823,23 @@
     <row r="110">
       <c r="A110" s="7" t="inlineStr">
         <is>
-          <t>Sofia Boldrini</t>
+          <t>Sofia Venturi</t>
         </is>
       </c>
       <c r="B110" s="8" t="inlineStr">
         <is>
-          <t>10ª Fase</t>
+          <t>7ª Fase</t>
         </is>
       </c>
       <c r="C110" s="8" t="n">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="D110" s="9">
         <f>IF(C110="","",C110/39)</f>
         <v/>
       </c>
       <c r="E110" s="8" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="F110" s="9">
         <f>IF(E110="","",E110/60)</f>
@@ -95854,7 +95858,7 @@
     <row r="111">
       <c r="A111" s="10" t="inlineStr">
         <is>
-          <t>Sofia Venturi</t>
+          <t>Suelen Dias Clasen</t>
         </is>
       </c>
       <c r="B111" s="11" t="inlineStr">
@@ -95863,14 +95867,14 @@
         </is>
       </c>
       <c r="C111" s="11" t="n">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="D111" s="12">
         <f>IF(C111="","",C111/39)</f>
         <v/>
       </c>
       <c r="E111" s="11" t="n">
-        <v>30</v>
+        <v>41</v>
       </c>
       <c r="F111" s="12">
         <f>IF(E111="","",E111/60)</f>
@@ -95889,23 +95893,23 @@
     <row r="112">
       <c r="A112" s="7" t="inlineStr">
         <is>
-          <t>Suelen Dias Clasen</t>
+          <t>Taina Farias</t>
         </is>
       </c>
       <c r="B112" s="8" t="inlineStr">
         <is>
-          <t>7ª Fase</t>
+          <t>11ª Fase</t>
         </is>
       </c>
       <c r="C112" s="8" t="n">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="D112" s="9">
         <f>IF(C112="","",C112/39)</f>
         <v/>
       </c>
       <c r="E112" s="8" t="n">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="F112" s="9">
         <f>IF(E112="","",E112/60)</f>
@@ -95924,23 +95928,23 @@
     <row r="113">
       <c r="A113" s="10" t="inlineStr">
         <is>
-          <t>Taina Farias</t>
+          <t>Tassiane Thaisi Thiesen</t>
         </is>
       </c>
       <c r="B113" s="11" t="inlineStr">
         <is>
-          <t>11ª Fase</t>
+          <t>10ª Fase</t>
         </is>
       </c>
       <c r="C113" s="11" t="n">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D113" s="12">
         <f>IF(C113="","",C113/39)</f>
         <v/>
       </c>
       <c r="E113" s="11" t="n">
-        <v>32</v>
+        <v>44</v>
       </c>
       <c r="F113" s="12">
         <f>IF(E113="","",E113/60)</f>
@@ -95959,16 +95963,16 @@
     <row r="114">
       <c r="A114" s="7" t="inlineStr">
         <is>
-          <t>Tassiane Thaisi Thiesen</t>
+          <t>Taís Cristina Paludo</t>
         </is>
       </c>
       <c r="B114" s="8" t="inlineStr">
         <is>
-          <t>10ª Fase</t>
+          <t>11ª Fase</t>
         </is>
       </c>
       <c r="C114" s="8" t="n">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="D114" s="9">
         <f>IF(C114="","",C114/39)</f>
@@ -95994,23 +95998,23 @@
     <row r="115">
       <c r="A115" s="10" t="inlineStr">
         <is>
-          <t>Taís Cristina Paludo</t>
+          <t>Tharik Stache Ribeiro</t>
         </is>
       </c>
       <c r="B115" s="11" t="inlineStr">
         <is>
-          <t>11ª Fase</t>
+          <t>6ª Fase</t>
         </is>
       </c>
       <c r="C115" s="11" t="n">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="D115" s="12">
         <f>IF(C115="","",C115/39)</f>
         <v/>
       </c>
       <c r="E115" s="11" t="n">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="F115" s="12">
         <f>IF(E115="","",E115/60)</f>
@@ -96029,7 +96033,7 @@
     <row r="116">
       <c r="A116" s="7" t="inlineStr">
         <is>
-          <t>Tharik Stache Ribeiro</t>
+          <t>Thiago Matheussi Alves</t>
         </is>
       </c>
       <c r="B116" s="8" t="inlineStr">
@@ -96038,14 +96042,14 @@
         </is>
       </c>
       <c r="C116" s="8" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D116" s="9">
         <f>IF(C116="","",C116/39)</f>
         <v/>
       </c>
       <c r="E116" s="8" t="n">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="F116" s="9">
         <f>IF(E116="","",E116/60)</f>
@@ -96064,7 +96068,7 @@
     <row r="117">
       <c r="A117" s="10" t="inlineStr">
         <is>
-          <t>Thiago Matheussi Alves</t>
+          <t>Thiago Robert Brito de Lima</t>
         </is>
       </c>
       <c r="B117" s="11" t="inlineStr">
@@ -96073,14 +96077,14 @@
         </is>
       </c>
       <c r="C117" s="11" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D117" s="12">
         <f>IF(C117="","",C117/39)</f>
         <v/>
       </c>
       <c r="E117" s="11" t="n">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="F117" s="12">
         <f>IF(E117="","",E117/60)</f>
@@ -96099,7 +96103,7 @@
     <row r="118">
       <c r="A118" s="7" t="inlineStr">
         <is>
-          <t>Thiago Robert Brito de Lima</t>
+          <t>Victor Hugo Tonet</t>
         </is>
       </c>
       <c r="B118" s="8" t="inlineStr">
@@ -96108,14 +96112,14 @@
         </is>
       </c>
       <c r="C118" s="8" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D118" s="9">
         <f>IF(C118="","",C118/39)</f>
         <v/>
       </c>
       <c r="E118" s="8" t="n">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="F118" s="9">
         <f>IF(E118="","",E118/60)</f>
@@ -96134,23 +96138,23 @@
     <row r="119">
       <c r="A119" s="10" t="inlineStr">
         <is>
-          <t>Victor Hugo Tonet</t>
+          <t>Victória Gabriela Wetzstein</t>
         </is>
       </c>
       <c r="B119" s="11" t="inlineStr">
         <is>
-          <t>6ª Fase</t>
+          <t>7ª Fase</t>
         </is>
       </c>
       <c r="C119" s="11" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="D119" s="12">
         <f>IF(C119="","",C119/39)</f>
         <v/>
       </c>
       <c r="E119" s="11" t="n">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="F119" s="12">
         <f>IF(E119="","",E119/60)</f>
@@ -96169,23 +96173,23 @@
     <row r="120">
       <c r="A120" s="7" t="inlineStr">
         <is>
-          <t>Victória Gabriela Wetzstein</t>
+          <t>Yasmin Minatti</t>
         </is>
       </c>
       <c r="B120" s="8" t="inlineStr">
         <is>
-          <t>7ª Fase</t>
+          <t>11ª Fase</t>
         </is>
       </c>
       <c r="C120" s="8" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="D120" s="9">
         <f>IF(C120="","",C120/39)</f>
         <v/>
       </c>
       <c r="E120" s="8" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F120" s="9">
         <f>IF(E120="","",E120/60)</f>
@@ -96204,7 +96208,7 @@
     <row r="121">
       <c r="A121" s="10" t="inlineStr">
         <is>
-          <t>Yasmin Minatti</t>
+          <t>Yasmin Paes Turnes</t>
         </is>
       </c>
       <c r="B121" s="11" t="inlineStr">
@@ -96213,14 +96217,14 @@
         </is>
       </c>
       <c r="C121" s="11" t="n">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="D121" s="12">
         <f>IF(C121="","",C121/39)</f>
         <v/>
       </c>
       <c r="E121" s="11" t="n">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="F121" s="12">
         <f>IF(E121="","",E121/60)</f>
@@ -96239,23 +96243,23 @@
     <row r="122">
       <c r="A122" s="7" t="inlineStr">
         <is>
-          <t>Yasmin Paes Turnes</t>
+          <t>Yasmin Primel Paludo</t>
         </is>
       </c>
       <c r="B122" s="8" t="inlineStr">
         <is>
-          <t>11ª Fase</t>
+          <t>10ª Fase</t>
         </is>
       </c>
       <c r="C122" s="8" t="n">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="D122" s="9">
         <f>IF(C122="","",C122/39)</f>
         <v/>
       </c>
       <c r="E122" s="8" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F122" s="9">
         <f>IF(E122="","",E122/60)</f>
@@ -96274,23 +96278,21 @@
     <row r="123">
       <c r="A123" s="10" t="inlineStr">
         <is>
-          <t>Yasmin Primel Paludo</t>
+          <t>Yasmin Rafaela Braun</t>
         </is>
       </c>
       <c r="B123" s="11" t="inlineStr">
         <is>
-          <t>10ª Fase</t>
-        </is>
-      </c>
-      <c r="C123" s="11" t="n">
-        <v>26</v>
-      </c>
+          <t>11ª Fase</t>
+        </is>
+      </c>
+      <c r="C123" s="11" t="n"/>
       <c r="D123" s="12">
         <f>IF(C123="","",C123/39)</f>
         <v/>
       </c>
       <c r="E123" s="11" t="n">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="F123" s="12">
         <f>IF(E123="","",E123/60)</f>
@@ -96302,28 +96304,30 @@
       </c>
       <c r="H123" s="10" t="inlineStr">
         <is>
-          <t>Nos dois simulados</t>
+          <t>Só no Simulado 02</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="7" t="inlineStr">
         <is>
-          <t>Yasmin Rafaela Braun</t>
+          <t>Élton Léo Junglos</t>
         </is>
       </c>
       <c r="B124" s="8" t="inlineStr">
         <is>
-          <t>11ª Fase</t>
-        </is>
-      </c>
-      <c r="C124" s="8" t="n"/>
+          <t>7ª Fase</t>
+        </is>
+      </c>
+      <c r="C124" s="8" t="n">
+        <v>17</v>
+      </c>
       <c r="D124" s="9">
         <f>IF(C124="","",C124/39)</f>
         <v/>
       </c>
       <c r="E124" s="8" t="n">
-        <v>34</v>
+        <v>19</v>
       </c>
       <c r="F124" s="9">
         <f>IF(E124="","",E124/60)</f>
@@ -96335,30 +96339,30 @@
       </c>
       <c r="H124" s="7" t="inlineStr">
         <is>
-          <t>Só no Simulado 02</t>
+          <t>Nos dois simulados</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="10" t="inlineStr">
         <is>
-          <t>Élton Léo Junglos</t>
+          <t>Émerson Roberto Bratz</t>
         </is>
       </c>
       <c r="B125" s="11" t="inlineStr">
         <is>
-          <t>7ª Fase</t>
+          <t>10ª Fase</t>
         </is>
       </c>
       <c r="C125" s="11" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="D125" s="12">
         <f>IF(C125="","",C125/39)</f>
         <v/>
       </c>
       <c r="E125" s="11" t="n">
-        <v>19</v>
+        <v>45</v>
       </c>
       <c r="F125" s="12">
         <f>IF(E125="","",E125/60)</f>
@@ -96377,23 +96381,23 @@
     <row r="126">
       <c r="A126" s="7" t="inlineStr">
         <is>
-          <t>Émerson Roberto Bratz</t>
+          <t>Íris Lyra Martendal</t>
         </is>
       </c>
       <c r="B126" s="8" t="inlineStr">
         <is>
-          <t>10ª Fase</t>
+          <t>7ª Fase</t>
         </is>
       </c>
       <c r="C126" s="8" t="n">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="D126" s="9">
         <f>IF(C126="","",C126/39)</f>
         <v/>
       </c>
       <c r="E126" s="8" t="n">
-        <v>45</v>
+        <v>29</v>
       </c>
       <c r="F126" s="9">
         <f>IF(E126="","",E126/60)</f>
@@ -96409,43 +96413,8 @@
         </is>
       </c>
     </row>
-    <row r="127">
-      <c r="A127" s="10" t="inlineStr">
-        <is>
-          <t>Íris Lyra Martendal</t>
-        </is>
-      </c>
-      <c r="B127" s="11" t="inlineStr">
-        <is>
-          <t>7ª Fase</t>
-        </is>
-      </c>
-      <c r="C127" s="11" t="n">
-        <v>16</v>
-      </c>
-      <c r="D127" s="12">
-        <f>IF(C127="","",C127/39)</f>
-        <v/>
-      </c>
-      <c r="E127" s="11" t="n">
-        <v>29</v>
-      </c>
-      <c r="F127" s="12">
-        <f>IF(E127="","",E127/60)</f>
-        <v/>
-      </c>
-      <c r="G127" s="19">
-        <f>IF(OR(C127="",E127=""),"",(F127-D127)*100)</f>
-        <v/>
-      </c>
-      <c r="H127" s="10" t="inlineStr">
-        <is>
-          <t>Nos dois simulados</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:H127"/>
+  <autoFilter ref="A1:H126"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Substitui gabarito deduzido do S02 pelo oficial e registra erros de chave
O gabarito oficial do Simulado 02 chegou e confere nas 60 questoes com o
que havia sido deduzido do cruzamento entre imagens e graficos - zero
divergencias. A deducao deixa de ser ressalva.

Registra no Leia-me duas provaveis falhas de chave, encontradas na
auditoria de itens em que um distrator vence o gabarito nas quatro fases:
Q17 do S01 (oficial C, 88-94% marcaram B) e Q59 do S02 (oficial B, 57-90%
marcaram C). Os numeros seguem reproduzindo a chave oficial.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KJtXaVvEGRV3wqA1hqbBYb
</commit_message>
<xml_diff>
--- a/dados/Dados_Simulados_MED_ENAMED_2026.xlsx
+++ b/dados/Dados_Simulados_MED_ENAMED_2026.xlsx
@@ -533,7 +533,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -646,122 +646,146 @@
     <row r="11" ht="52" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Ressalva 3 — Gabarito do S02</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>O PDF do Simulado 02 vem com a folha de gabarito em branco. O gabarito das 60 questões foi deduzido cruzando o cache dos gráficos com as % das imagens: em todas as 60 questões uma única alternativa reproduz a % de acerto simultaneamente nas 4 fases, e o resultado fecha com a soma de acertos dos alunos. Gabarito deduzido: DBCCCDCBDADCBABBACCBACDCBADABBACADABAABCCDCBABBCADCCEEBDEDBC</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="91" customHeight="1">
+          <t>Gabarito do S02 — conferido</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>A folha de gabarito vinha em branco no PDF da prova, então as 60 respostas foram deduzidas cruzando o cache dos gráficos com as % das imagens. O gabarito oficial foi obtido depois e confere nas 60 questões, sem nenhuma divergência. Deixou de ser dedução: DBCCCDCBDADCBABBACCBACDCBADABBACADABAABCCDCBABBCADCCEEBDEDBC</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="52" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
+          <t>Ressalva 3 — Q17 do S01</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Não é problema de extração, é da prova. O gabarito oficial marca C, que descreve 'pontos de atenção à saúde' (a definição usada na Q01); a alternativa B é a que define Atenção Primária. Entre 88% e 94% dos alunos marcaram B e foram contados como erro. Corrigir a chave elevaria a média de todas as fases em cerca de 2 p.p. Os números aqui reproduzem o dashboard, com C.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="39" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Ressalva 3b — Q59 do S02</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Mesma situação: o gabarito oficial marca B, que manda o paciente em crise aguardar o técnico de referência; a alternativa C descreve a conduta de acolhimento à crise no CAPS. De 57% a 90% dos alunos marcaram C. Corrigir elevaria as médias entre 0,7 e 1,5 p.p. Reproduzido aqui como B.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="91" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
           <t>Ressalva 4 — nomes</t>
         </is>
       </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>Os 126 nomes foram lidos duas vezes de forma independente (uma imagem por simulado) e 112 coincidem caractere a caractere, o que confirma essa leitura. Três casos exigiram intervenção: 'Lucas Eduardo dos Santos Vian…' e 'Maria Eduarda Medeiros Macha…' estavam truncados na imagem da 10ª Fase do Simulado 01 e foram completados pela lista do Simulado 02; e 'Maria Amélia Vozniak Deluca' (S01) e 'Maria Amélia Vozniak Deluca Schneider' (S02) são a mesma aluna, unificadas na aba de comparativo. Os 13 nomes restantes que aparecem em um só simulado são mudanças reais de turma (a 11ª Fase perdeu 4 alunos e ganhou 6 entre as duas aplicações).</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="15" customHeight="1">
-      <c r="A13" s="2" t="inlineStr"/>
-      <c r="B13" s="3" t="inlineStr"/>
-    </row>
-    <row r="14" ht="15" customHeight="1">
-      <c r="A14" s="4" t="inlineStr">
+    <row r="15" ht="15" customHeight="1">
+      <c r="A15" s="2" t="inlineStr"/>
+      <c r="B15" s="3" t="inlineStr"/>
+    </row>
+    <row r="16" ht="15" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>Abas</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr"/>
-    </row>
-    <row r="15" ht="15" customHeight="1">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Alunos</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>Uma linha por aluno por simulado: fase, acertos, % e posição.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="15" customHeight="1">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Questões</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>Uma linha por questão: gabarito e acertos/% por fase, % geral e dificuldade.</t>
-        </is>
-      </c>
+      <c r="B16" s="3" t="inlineStr"/>
     </row>
     <row r="17" ht="15" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Questão x Fase</t>
+          <t xml:space="preserve">  Alunos</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Mesma informação em formato longo, pronta para tabela dinâmica.</t>
+          <t>Uma linha por aluno por simulado: fase, acertos, % e posição.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Distribuição respostas</t>
+          <t xml:space="preserve">  Questões</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Nº e % de alunos em cada alternativa A–E, por questão e por fase.</t>
+          <t>Uma linha por questão: gabarito e acertos/% por fase, % geral e dificuldade.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Resumo por fase</t>
+          <t xml:space="preserve">  Questão x Fase</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Estatísticas descritivas de cada fase em cada simulado.</t>
+          <t>Mesma informação em formato longo, pronta para tabela dinâmica.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Distribuição respostas</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Nº e % de alunos em cada alternativa A–E, por questão e por fase.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="15" customHeight="1">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Resumo por fase</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Estatísticas descritivas de cada fase em cada simulado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="15" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">  Comparativo S01 x S02</t>
         </is>
       </c>
-      <c r="B20" s="3" t="inlineStr">
+      <c r="B22" s="3" t="inlineStr">
         <is>
           <t>Alunos presentes nos dois simulados e variação em pontos percentuais.</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="15" customHeight="1">
-      <c r="A21" s="2" t="inlineStr"/>
-      <c r="B21" s="3" t="inlineStr"/>
-    </row>
-    <row r="22" ht="15" customHeight="1">
-      <c r="A22" s="4" t="inlineStr">
+    <row r="23" ht="15" customHeight="1">
+      <c r="A23" s="2" t="inlineStr"/>
+      <c r="B23" s="3" t="inlineStr"/>
+    </row>
+    <row r="24" ht="15" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
         <is>
           <t>Observação</t>
         </is>
       </c>
-      <c r="B22" s="3" t="inlineStr">
+      <c r="B24" s="3" t="inlineStr">
         <is>
           <t>Percentuais são fórmulas sobre as contagens; ao alterar um número de acertos, o resto recalcula.</t>
         </is>

</xml_diff>